<commit_message>
updated new corpora from student projects AY2025sem2 and rerun scripts
</commit_message>
<xml_diff>
--- a/scripts/checks/results/HLR_results_01_Dunn_lgs_tPBC.xlsx
+++ b/scripts/checks/results/HLR_results_01_Dunn_lgs_tPBC.xlsx
@@ -562,57 +562,57 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2773093265883012</v>
+        <v>0.2778077214292567</v>
       </c>
       <c r="H2" t="n">
-        <v>45.27870877721755</v>
+        <v>45.39138966360625</v>
       </c>
       <c r="I2" t="n">
-        <v>6.498545364230793e-10</v>
+        <v>6.23405371411057e-10</v>
       </c>
       <c r="J2" t="n">
-        <v>17.9167062783317</v>
+        <v>17.90435023956635</v>
       </c>
       <c r="K2" t="n">
         <v>24.79166666666667</v>
       </c>
       <c r="L2" t="n">
-        <v>6.874960388334969</v>
+        <v>6.887316427100323</v>
       </c>
       <c r="M2" t="n">
-        <v>0.151836493884167</v>
+        <v>0.1517317816912402</v>
       </c>
       <c r="N2" t="n">
         <v>0.2083333333333334</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>{'const': 0.7704480129557647, 'N1ratio-ArgsPreds': -3.197547552292713}</t>
+          <t>{'const': 0.7491199802103012, 'N1ratio-ArgsPreds': -3.0224806007943616}</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>{'const': 1.1179374076442262e-16, 'N1ratio-ArgsPreds': 6.498545364231103e-10}</t>
+          <t>{'const': 6.899475278910947e-17, 'N1ratio-ArgsPreds': 6.234053714110714e-10}</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.5266016773504437}</t>
+          <t>{'N1ratio-ArgsPreds': -0.5270746829712618}</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5266016773504444)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5270746829712628)}</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5266016773504445)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5270746829712628)}</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(27.730932658830167)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(27.78077214292572)}</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -641,67 +641,67 @@
         <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4435495458492533</v>
+        <v>0.4518731968028366</v>
       </c>
       <c r="H3" t="n">
-        <v>46.63065370623617</v>
+        <v>48.22712893946424</v>
       </c>
       <c r="I3" t="n">
-        <v>1.280708583570932e-15</v>
+        <v>5.303234199251507e-16</v>
       </c>
       <c r="J3" t="n">
-        <v>13.7953341758206</v>
+        <v>13.58897699592968</v>
       </c>
       <c r="K3" t="n">
         <v>24.79166666666667</v>
       </c>
       <c r="L3" t="n">
-        <v>5.498166245423037</v>
+        <v>5.601344835368496</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1179088391095778</v>
+        <v>0.1161451025293135</v>
       </c>
       <c r="N3" t="n">
         <v>0.2083333333333334</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{'const': 0.36971985752381675, 'N1ratio-ArgsPreds': -2.873540181419574, 'Macro_class': 0.1329106641396056}</t>
+          <t>{'const': 0.3495411554324628, 'N1ratio-ArgsPreds': -2.757925732377074, 'Macro_class': 0.13567485618445077}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>{'const': 0.00023828960396245433, 'N1ratio-ArgsPreds': 4.587359490291268e-10, 'Macro_class': 3.414209397804697e-08}</t>
+          <t>{'const': 0.00029957870029502775, 'N1ratio-ArgsPreds': 1.866479010578518e-10, 'Macro_class': 1.4401635797998425e-08}</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.47324114957553637, 'Macro_class': 0.4112025841180598}</t>
+          <t>{'N1ratio-ArgsPreds': -0.4809403344619948, 'Macro_class': 0.4197545157421846}</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.532458628316241), 'Macro_class': np.float64(0.47961397213721435)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5424294947827045), 'Macro_class': np.float64(0.49094167482766166)}</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4692396659420063), 'Macro_class': np.float64(0.4077256666693338)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4780266886345877), 'Macro_class': np.float64(0.4172115475074733)}</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(22.018586409336567), 'Macro_class': np.float64(16.62402192609527)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(22.850951504694905), 'Macro_class': np.float64(17.406547537358065)}</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.1662402192609521</v>
+        <v>0.1740654753735799</v>
       </c>
       <c r="V3" t="n">
-        <v>34.95388584634386</v>
+        <v>37.15501686821039</v>
       </c>
       <c r="W3" t="n">
-        <v>3.414209397805013e-08</v>
+        <v>1.440163579800052e-08</v>
       </c>
     </row>
     <row r="4">
@@ -726,67 +726,67 @@
         <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4438874979987454</v>
+        <v>0.4524291368054834</v>
       </c>
       <c r="H4" t="n">
-        <v>30.86362896150001</v>
+        <v>31.9482423171426</v>
       </c>
       <c r="I4" t="n">
-        <v>9.65099385607767e-15</v>
+        <v>3.968843394245544e-15</v>
       </c>
       <c r="J4" t="n">
-        <v>13.78695577878111</v>
+        <v>13.57519431669739</v>
       </c>
       <c r="K4" t="n">
         <v>24.79166666666667</v>
       </c>
       <c r="L4" t="n">
-        <v>3.668236962628522</v>
+        <v>3.738824116656426</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1188530670584578</v>
+        <v>0.1170275372129086</v>
       </c>
       <c r="N4" t="n">
         <v>0.2083333333333334</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>{'const': 0.3924579532958908, 'N1ratio-ArgsPreds': -2.8633566408845166, 'Macro_class': 0.12862378502348312, 'Fam_class': -0.0002931873723604867}</t>
+          <t>{'const': 0.37909096371719414, 'N1ratio-ArgsPreds': -2.74734323219882, 'Macro_class': 0.13015781114532332, 'Fam_class': -0.00037564029680614303}</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>{'const': 0.0031357338238347967, 'N1ratio-ArgsPreds': 6.948974056809461e-10, 'Macro_class': 9.421112468682298e-06, 'Fam_class': 0.791090525642769}</t>
+          <t>{'const': 0.003603053297576945, 'N1ratio-ArgsPreds': 2.7802816721337533e-10, 'Macro_class': 6.412880396543444e-06, 'Fam_class': 0.7320837246068297}</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.47156403002080693, 'Macro_class': 0.3979397223171457, 'Fam_class': -0.022856974924660392}</t>
+          <t>{'N1ratio-ArgsPreds': -0.47909490725725756, 'Macro_class': 0.4026857335532548, 'Fam_class': -0.029285029486990098}</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5296671694901757), 'Macro_class': np.float64(0.39529044010156983), 'Fam_class': np.float64(-0.02464417907642201)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5399979456643242), 'Macro_class': np.float64(0.4020070160305793), 'Fam_class': np.float64(-0.03184736040668646)}</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.46567536520218356), 'Macro_class': np.float64(0.32091640171694724), 'Fam_class': np.float64(-0.018383474902530714)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4747580273812399), 'Macro_class': np.float64(0.324885748041981), 'Fam_class': np.float64(-0.023578379983510613)}</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(21.685354575618703), 'Macro_class': np.float64(10.298733689095306), 'Fam_class': np.float64(0.03379521494919766)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(22.539518456292612), 'Macro_class': np.float64(10.555074928079756), 'Fam_class': np.float64(0.0555940002646814)}</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>0.0003379521494920601</v>
+        <v>0.0005559400026468042</v>
       </c>
       <c r="V4" t="n">
-        <v>0.07049373858707195</v>
+        <v>0.1177729580620883</v>
       </c>
       <c r="W4" t="n">
-        <v>0.7910905256429911</v>
+        <v>0.7320837246068701</v>
       </c>
     </row>
     <row r="5">
@@ -811,67 +811,67 @@
         <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4619214611791157</v>
+        <v>0.4641730366459158</v>
       </c>
       <c r="H5" t="n">
-        <v>19.57299642160541</v>
+        <v>19.75105016977905</v>
       </c>
       <c r="I5" t="n">
-        <v>4.924562337235511e-14</v>
+        <v>3.904950328100897e-14</v>
       </c>
       <c r="J5" t="n">
-        <v>13.33986377493443</v>
+        <v>13.28404346648667</v>
       </c>
       <c r="K5" t="n">
         <v>24.79166666666667</v>
       </c>
       <c r="L5" t="n">
-        <v>2.290360578346449</v>
+        <v>2.301524640035999</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1170163489029336</v>
+        <v>0.1165266970744445</v>
       </c>
       <c r="N5" t="n">
         <v>0.2083333333333334</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>{'const': 0.17547142028805868, 'N1ratio-ArgsPreds': -2.985367830583762, 'Macro_class': 0.1203900883589171, 'Fam_class': -0.0013547988832423045, 'Nlen_freq': 0.7918523166300422, 'Vlen_freq': -0.0543043407850019}</t>
+          <t>{'const': 0.19847538662571965, 'N1ratio-ArgsPreds': -2.811994104422621, 'Macro_class': 0.12455445172274414, 'Fam_class': -0.0012336323262047975, 'Nlen_freq': 0.5644678913695322, 'Vlen_freq': 0.04541726352754072}</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>{'const': 0.3187166717733552, 'N1ratio-ArgsPreds': 3.867429991603257e-10, 'Macro_class': 3.336160483729077e-05, 'Fam_class': 0.27046341802115037, 'Nlen_freq': 0.13000228580547257, 'Vlen_freq': 0.9136473251109488}</t>
+          <t>{'const': 0.2544954253059988, 'N1ratio-ArgsPreds': 3.305864394821834e-10, 'Macro_class': 1.6779219729318443e-05, 'Fam_class': 0.31405876759070767, 'Nlen_freq': 0.269804779604789, 'Vlen_freq': 0.9267919252118344}</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.49165796016582575, 'Macro_class': 0.37246609033109573, 'Fam_class': -0.10562052469351396, 'Nlen_freq': 0.16159289070001517, 'Vlen_freq': -0.01067839295176575}</t>
+          <t>{'N1ratio-ArgsPreds': -0.49036903684876587, 'Macro_class': 0.3853499096054739, 'Fam_class': -0.09617434379692162, 'Nlen_freq': 0.11764332488741701, 'Vlen_freq': 0.009085055355778787}</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5402577251965031), 'Macro_class': np.float64(0.37514083559807176), 'Fam_class': np.float64(-0.10316169926315122), 'Nlen_freq': np.float64(0.1414039763691345), 'Vlen_freq': np.float64(-0.010178292348936926)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5420208744613125), 'Macro_class': np.float64(0.3880384897849444), 'Fam_class': np.float64(-0.09428630984713471), 'Nlen_freq': np.float64(0.10330288117179962), 'Vlen_freq': np.float64(0.008624253891698224)}</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.47094468826045766), 'Macro_class': np.float64(0.2968605689357376), 'Fam_class': np.float64(-0.07607897649656697), 'Nlen_freq': np.float64(0.10477805456946081), 'Vlen_freq': np.float64(-0.00746655473774999)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.47212861844772075), 'Macro_class': np.float64(0.3081940707749217), 'Fam_class': np.float64(-0.06932661118839695), 'Nlen_freq': np.float64(0.07602465413582278), 'Vlen_freq': np.float64(0.006313206090882815)}</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(22.178889940073965), 'Macro_class': np.float64(8.81261973888498), 'Fam_class': np.float64(0.5788010664765191), 'Nlen_freq': np.float64(1.0978440719360907), 'Vlen_freq': np.float64(0.005574943965181683)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(22.29054323573535), 'Macro_class': np.float64(9.498358526081747), 'Fam_class': np.float64(0.48061790188671644), 'Nlen_freq': np.float64(0.5779748036471476), 'Vlen_freq': np.float64(0.003985657114595988)}</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0.01803396318037032</v>
+        <v>0.01174389984043245</v>
       </c>
       <c r="V5" t="n">
-        <v>1.910382643272988</v>
+        <v>1.249288178247753</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1527325792761629</v>
+        <v>0.2906037998719303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
use updated annotations before base datasets
</commit_message>
<xml_diff>
--- a/scripts/checks/results/HLR_results_01_Dunn_lgs_tPBC.xlsx
+++ b/scripts/checks/results/HLR_results_01_Dunn_lgs_tPBC.xlsx
@@ -562,57 +562,57 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2778077214292567</v>
+        <v>0.2755848639634494</v>
       </c>
       <c r="H2" t="n">
-        <v>45.39138966360625</v>
+        <v>44.89002552542782</v>
       </c>
       <c r="I2" t="n">
-        <v>6.23405371411057e-10</v>
+        <v>7.501800790435129e-10</v>
       </c>
       <c r="J2" t="n">
-        <v>17.90435023956635</v>
+        <v>17.95945858090615</v>
       </c>
       <c r="K2" t="n">
         <v>24.79166666666667</v>
       </c>
       <c r="L2" t="n">
-        <v>6.887316427100323</v>
+        <v>6.832208085760517</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1517317816912402</v>
+        <v>0.152198801533103</v>
       </c>
       <c r="N2" t="n">
         <v>0.2083333333333334</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>{'const': 0.7491199802103012, 'N1ratio-ArgsPreds': -3.0224806007943616}</t>
+          <t>{'const': 0.7461726021992878, 'N1ratio-ArgsPreds': -3.0029926664449578}</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>{'const': 6.899475278910947e-17, 'N1ratio-ArgsPreds': 6.234053714110714e-10}</t>
+          <t>{'const': 8.338478385942126e-17, 'N1ratio-ArgsPreds': 7.501800790435231e-10}</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.5270746829712618}</t>
+          <t>{'N1ratio-ArgsPreds': -0.5249617738116265}</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5270746829712628)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5249617738116272)}</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5270746829712628)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5249617738116275)}</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(27.78077214292572)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(27.558486396345028)}</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -641,67 +641,67 @@
         <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4518731968028366</v>
+        <v>0.4501391091355157</v>
       </c>
       <c r="H3" t="n">
-        <v>48.22712893946424</v>
+        <v>47.89054526687111</v>
       </c>
       <c r="I3" t="n">
-        <v>5.303234199251507e-16</v>
+        <v>6.379558655543208e-16</v>
       </c>
       <c r="J3" t="n">
-        <v>13.58897699592968</v>
+        <v>13.63196791934868</v>
       </c>
       <c r="K3" t="n">
         <v>24.79166666666667</v>
       </c>
       <c r="L3" t="n">
-        <v>5.601344835368496</v>
+        <v>5.579849373658997</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1161451025293135</v>
+        <v>0.1165125463192195</v>
       </c>
       <c r="N3" t="n">
         <v>0.2083333333333334</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>{'const': 0.3495411554324628, 'N1ratio-ArgsPreds': -2.757925732377074, 'Macro_class': 0.13567485618445077}</t>
+          <t>{'const': 0.3464291616403392, 'N1ratio-ArgsPreds': -2.740491741401292, 'Macro_class': 0.13585421272097262}</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>{'const': 0.00029957870029502775, 'N1ratio-ArgsPreds': 1.866479010578518e-10, 'Macro_class': 1.4401635797998425e-08}</t>
+          <t>{'const': 0.00033733229968009, 'N1ratio-ArgsPreds': 2.253411481444149e-10, 'Macro_class': 1.4475646756260623e-08}</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.4809403344619948, 'Macro_class': 0.4197545157421846}</t>
+          <t>{'N1ratio-ArgsPreds': -0.47907323309758887, 'Macro_class': 0.4203094138143121}</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5424294947827045), 'Macro_class': np.float64(0.49094167482766166)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5403674108051154), 'Macro_class': np.float64(0.4908756051788926)}</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4780266886345877), 'Macro_class': np.float64(0.4172115475074733)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.47620943646638075), 'Macro_class': np.float64(0.4177968946414836)}</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(22.850951504694905), 'Macro_class': np.float64(17.406547537358065)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(22.677542737962792), 'Macro_class': np.float64(17.455424517206698)}</t>
         </is>
       </c>
       <c r="U3" t="n">
-        <v>0.1740654753735799</v>
+        <v>0.1745542451720663</v>
       </c>
       <c r="V3" t="n">
-        <v>37.15501686821039</v>
+        <v>37.14184264500648</v>
       </c>
       <c r="W3" t="n">
-        <v>1.440163579800052e-08</v>
+        <v>1.447564675626127e-08</v>
       </c>
     </row>
     <row r="4">
@@ -726,67 +726,67 @@
         <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4524291368054834</v>
+        <v>0.4506642630178418</v>
       </c>
       <c r="H4" t="n">
-        <v>31.9482423171426</v>
+        <v>31.72137485978971</v>
       </c>
       <c r="I4" t="n">
-        <v>3.968843394245544e-15</v>
+        <v>4.774220202953495e-15</v>
       </c>
       <c r="J4" t="n">
-        <v>13.57519431669739</v>
+        <v>13.61894847934934</v>
       </c>
       <c r="K4" t="n">
         <v>24.79166666666667</v>
       </c>
       <c r="L4" t="n">
-        <v>3.738824116656426</v>
+        <v>3.724239395772444</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1170275372129086</v>
+        <v>0.1174047282702529</v>
       </c>
       <c r="N4" t="n">
         <v>0.2083333333333334</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>{'const': 0.37909096371719414, 'N1ratio-ArgsPreds': -2.74734323219882, 'Macro_class': 0.13015781114532332, 'Fam_class': -0.00037564029680614303}</t>
+          <t>{'const': 0.37512056148652373, 'N1ratio-ArgsPreds': -2.7300076802617337, 'Macro_class': 0.1304923364381657, 'Fam_class': -0.0003651399539774488}</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>{'const': 0.003603053297576945, 'N1ratio-ArgsPreds': 2.7802816721337533e-10, 'Macro_class': 6.412880396543444e-06, 'Fam_class': 0.7320837246068297}</t>
+          <t>{'const': 0.003969640655784507, 'N1ratio-ArgsPreds': 3.3632666003065255e-10, 'Macro_class': 6.285648886347259e-06, 'Fam_class': 0.7397301091874162}</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.47909490725725756, 'Macro_class': 0.4026857335532548, 'Fam_class': -0.029285029486990098}</t>
+          <t>{'N1ratio-ArgsPreds': -0.47724048425538557, 'Macro_class': 0.4037206968931803, 'Fam_class': -0.028466419630762376}</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5399979456643242), 'Macro_class': np.float64(0.4020070160305793), 'Fam_class': np.float64(-0.03184736040668646)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.5378796636221189), 'Macro_class': np.float64(0.4023529757543716), 'Fam_class': np.float64(-0.03090415508525273)}</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.4747580273812399), 'Macro_class': np.float64(0.324885748041981), 'Fam_class': np.float64(-0.023578379983510613)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.4728956658453139), 'Macro_class': np.float64(0.3257430010658656), 'Fam_class': np.float64(-0.022916236216408228)}</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(22.539518456292612), 'Macro_class': np.float64(10.555074928079756), 'Fam_class': np.float64(0.0555940002646814)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(22.363031077528277), 'Macro_class': np.float64(10.610850274339652), 'Fam_class': np.float64(0.05251538823262201)}</t>
         </is>
       </c>
       <c r="U4" t="n">
-        <v>0.0005559400026468042</v>
+        <v>0.0005251538823261015</v>
       </c>
       <c r="V4" t="n">
-        <v>0.1177729580620883</v>
+        <v>0.1108936598308482</v>
       </c>
       <c r="W4" t="n">
-        <v>0.7320837246068701</v>
+        <v>0.7397301091873982</v>
       </c>
     </row>
     <row r="5">
@@ -811,67 +811,67 @@
         <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4641730366459158</v>
+        <v>0.462078080803026</v>
       </c>
       <c r="H5" t="n">
-        <v>19.75105016977905</v>
+        <v>19.5853336075922</v>
       </c>
       <c r="I5" t="n">
-        <v>3.904950328100897e-14</v>
+        <v>4.845893345739595e-14</v>
       </c>
       <c r="J5" t="n">
-        <v>13.28404346648667</v>
+        <v>13.33598091342498</v>
       </c>
       <c r="K5" t="n">
         <v>24.79166666666667</v>
       </c>
       <c r="L5" t="n">
-        <v>2.301524640035999</v>
+        <v>2.291137150648338</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1165266970744445</v>
+        <v>0.1169822887142542</v>
       </c>
       <c r="N5" t="n">
         <v>0.2083333333333334</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>{'const': 0.19847538662571965, 'N1ratio-ArgsPreds': -2.811994104422621, 'Macro_class': 0.12455445172274414, 'Fam_class': -0.0012336323262047975, 'Nlen_freq': 0.5644678913695322, 'Vlen_freq': 0.04541726352754072}</t>
+          <t>{'const': 0.19756951482544696, 'N1ratio-ArgsPreds': -2.795406722501567, 'Macro_class': 0.12503015815205792, 'Fam_class': -0.0012117068858907174, 'Nlen_freq': 0.564849707929282, 'Vlen_freq': 0.04252843754088842}</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>{'const': 0.2544954253059988, 'N1ratio-ArgsPreds': 3.305864394821834e-10, 'Macro_class': 1.6779219729318443e-05, 'Fam_class': 0.31405876759070767, 'Nlen_freq': 0.269804779604789, 'Vlen_freq': 0.9267919252118344}</t>
+          <t>{'const': 0.25683082153920567, 'N1ratio-ArgsPreds': 4.1746888508307303e-10, 'Macro_class': 1.6155544701682485e-05, 'Fam_class': 0.3237652085441375, 'Nlen_freq': 0.27727178090953286, 'Vlen_freq': 0.931664121582828}</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': -0.49036903684876587, 'Macro_class': 0.3853499096054739, 'Fam_class': -0.09617434379692162, 'Nlen_freq': 0.11764332488741701, 'Vlen_freq': 0.009085055355778787}</t>
+          <t>{'N1ratio-ArgsPreds': -0.48867307868141446, 'Macro_class': 0.38682166293905096, 'Fam_class': -0.09446502993583596, 'Nlen_freq': 0.1164090427593988, 'Vlen_freq': 0.008518109158387573}</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.5420208744613125), 'Macro_class': np.float64(0.3880384897849444), 'Fam_class': np.float64(-0.09428630984713471), 'Nlen_freq': np.float64(0.10330288117179962), 'Vlen_freq': np.float64(0.008624253891698224)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.53939488036786), 'Macro_class': np.float64(0.3887338218876132), 'Fam_class': np.float64(-0.09242206766953988), 'Nlen_freq': np.float64(0.10171572002683264), 'Vlen_freq': np.float64(0.008048846234299935)}</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(-0.47212861844772075), 'Macro_class': np.float64(0.3081940707749217), 'Fam_class': np.float64(-0.06932661118839695), 'Nlen_freq': np.float64(0.07602465413582278), 'Vlen_freq': np.float64(0.006313206090882815)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(-0.46981517604417433), 'Macro_class': np.float64(0.3094477000622494), 'Fam_class': np.float64(-0.06807663880811016), 'Nlen_freq': np.float64(0.07499046134790832), 'Vlen_freq': np.float64(0.005903469439992617)}</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>{'N1ratio-ArgsPreds': np.float64(22.29054323573535), 'Macro_class': np.float64(9.498358526081747), 'Fam_class': np.float64(0.48061790188671644), 'Nlen_freq': np.float64(0.5779748036471476), 'Vlen_freq': np.float64(0.003985657114595988)}</t>
+          <t>{'N1ratio-ArgsPreds': np.float64(22.07262996414185), 'Macro_class': np.float64(9.575787907381587), 'Fam_class': np.float64(0.463442875140989), 'Nlen_freq': np.float64(0.5623569293172132), 'Vlen_freq': np.float64(0.003485095142892674)}</t>
         </is>
       </c>
       <c r="U5" t="n">
-        <v>0.01174389984043245</v>
+        <v>0.01141381778518424</v>
       </c>
       <c r="V5" t="n">
-        <v>1.249288178247753</v>
+        <v>1.209446186403258</v>
       </c>
       <c r="W5" t="n">
-        <v>0.2906037998719303</v>
+        <v>0.302161504198549</v>
       </c>
     </row>
   </sheetData>

</xml_diff>